<commit_message>
fix(login/emp-manager): achieve 100% pass rate across 22 tests and ensure summary popups display on completion
</commit_message>
<xml_diff>
--- a/shared/test_data/Swarajya-test-data.xlsx
+++ b/shared/test_data/Swarajya-test-data.xlsx
@@ -12846,17 +12846,15 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>360</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>test@1234</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Test@1010</t>
         </is>
       </c>
       <c r="E2" s="5" t="n">

</xml_diff>

<commit_message>
fix(shared): restore inject_session_storage, support sheet_name kwargs in login, add popup auto-close timeout, and sync staging 2FA auth code
</commit_message>
<xml_diff>
--- a/shared/test_data/Swarajya-test-data.xlsx
+++ b/shared/test_data/Swarajya-test-data.xlsx
@@ -1816,10 +1816,8 @@
           <t>test@1234</t>
         </is>
       </c>
-      <c r="M2" s="48" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
+      <c r="M2" s="48" t="n">
+        <v>111111</v>
       </c>
       <c r="N2" s="60" t="n"/>
       <c r="O2" s="60" t="n"/>
@@ -3798,10 +3796,8 @@
           <t>test@1234</t>
         </is>
       </c>
-      <c r="H2" s="48" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
+      <c r="H2" s="48" t="n">
+        <v>111111</v>
       </c>
       <c r="I2" s="60" t="n"/>
       <c r="J2" s="60" t="n"/>
@@ -4939,10 +4935,8 @@
           <t>test@1234</t>
         </is>
       </c>
-      <c r="I2" s="48" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
+      <c r="I2" s="48" t="n">
+        <v>111111</v>
       </c>
     </row>
     <row r="3">
@@ -13291,10 +13285,8 @@
           <t>test@1234</t>
         </is>
       </c>
-      <c r="I2" s="48" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
+      <c r="I2" s="48" t="n">
+        <v>111111</v>
       </c>
       <c r="J2" s="49" t="n"/>
       <c r="K2" s="49" t="n"/>
@@ -42638,10 +42630,8 @@
           <t>test@1234</t>
         </is>
       </c>
-      <c r="L2" s="48" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
+      <c r="L2" s="48" t="n">
+        <v>111111</v>
       </c>
       <c r="M2" s="49" t="n"/>
       <c r="N2" s="49" t="n"/>
@@ -44846,10 +44836,8 @@
           <t>test@1234</t>
         </is>
       </c>
-      <c r="F2" s="48" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
+      <c r="F2" s="48" t="n">
+        <v>111111</v>
       </c>
       <c r="G2" s="49" t="n"/>
       <c r="H2" s="49" t="n"/>
@@ -46089,10 +46077,8 @@
           <t>test@1234</t>
         </is>
       </c>
-      <c r="I2" s="48" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
+      <c r="I2" s="48" t="n">
+        <v>111111</v>
       </c>
       <c r="J2" s="60" t="n"/>
       <c r="K2" s="60" t="n"/>
@@ -47886,10 +47872,8 @@
           <t>test@1234</t>
         </is>
       </c>
-      <c r="H2" s="48" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
+      <c r="H2" s="48" t="n">
+        <v>111111</v>
       </c>
       <c r="I2" s="60" t="n"/>
       <c r="J2" s="60" t="n"/>
@@ -49149,7 +49133,7 @@
         </is>
       </c>
       <c r="I2" s="76" t="n">
-        <v>123456</v>
+        <v>111111</v>
       </c>
     </row>
     <row r="4" ht="27" customHeight="1" s="150">
@@ -50797,10 +50781,8 @@
           <t>test@1234</t>
         </is>
       </c>
-      <c r="G2" s="48" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
+      <c r="G2" s="48" t="n">
+        <v>111111</v>
       </c>
       <c r="H2" s="49" t="n"/>
       <c r="I2" s="49" t="n"/>

</xml_diff>

<commit_message>
fix(vendor-mgmt): eliminate false-alarm popup warnings, add mandatory fields and atomic excel save
</commit_message>
<xml_diff>
--- a/shared/test_data/Swarajya-test-data.xlsx
+++ b/shared/test_data/Swarajya-test-data.xlsx
@@ -44934,6 +44934,21 @@
           <t>Tax Number</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Vendor State</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Vendor POC</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>TDS Percentage (%)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="42" t="inlineStr">
@@ -44975,6 +44990,19 @@
         <v>30</v>
       </c>
       <c r="I5" s="31" t="n"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="34" t="inlineStr">
@@ -45016,6 +45044,19 @@
         <v>30</v>
       </c>
       <c r="I6" s="50" t="n"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="42" t="inlineStr">
@@ -45057,6 +45098,19 @@
         <v>30</v>
       </c>
       <c r="I7" s="31" t="n"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="34" t="inlineStr">
@@ -45098,6 +45152,19 @@
         <v>30</v>
       </c>
       <c r="I8" s="50" t="n"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="42" t="inlineStr">
@@ -45125,7 +45192,11 @@
           <t>+1-234-5678</t>
         </is>
       </c>
-      <c r="F9" s="31" t="n"/>
+      <c r="F9" s="31" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G9" s="31" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45133,6 +45204,19 @@
       </c>
       <c r="H9" s="31" t="n"/>
       <c r="I9" s="31" t="n"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="34" t="inlineStr">
@@ -45160,7 +45244,11 @@
           <t>+44-123-4567</t>
         </is>
       </c>
-      <c r="F10" s="50" t="n"/>
+      <c r="F10" s="50" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G10" s="50" t="inlineStr">
         <is>
           <t>Automated</t>
@@ -45168,6 +45256,19 @@
       </c>
       <c r="H10" s="50" t="n"/>
       <c r="I10" s="50" t="n"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="42" t="inlineStr">
@@ -45195,7 +45296,11 @@
           <t>+1-987-6543</t>
         </is>
       </c>
-      <c r="F11" s="31" t="n"/>
+      <c r="F11" s="31" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G11" s="31" t="inlineStr">
         <is>
           <t>Inactive</t>
@@ -45203,6 +45308,19 @@
       </c>
       <c r="H11" s="31" t="n"/>
       <c r="I11" s="31" t="n"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="34" t="inlineStr">
@@ -45230,7 +45348,11 @@
           <t>+1-000-0000</t>
         </is>
       </c>
-      <c r="F12" s="50" t="n"/>
+      <c r="F12" s="50" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G12" s="50" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45238,6 +45360,19 @@
       </c>
       <c r="H12" s="50" t="n"/>
       <c r="I12" s="50" t="n"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="42" t="inlineStr">
@@ -45265,7 +45400,11 @@
           <t>+1-987-6543</t>
         </is>
       </c>
-      <c r="F13" s="31" t="n"/>
+      <c r="F13" s="31" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G13" s="31" t="inlineStr">
         <is>
           <t>Inactive</t>
@@ -45273,6 +45412,19 @@
       </c>
       <c r="H13" s="31" t="n"/>
       <c r="I13" s="31" t="n"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="34" t="inlineStr">
@@ -45300,7 +45452,11 @@
           <t>+1-555-000-0000</t>
         </is>
       </c>
-      <c r="F14" s="50" t="n"/>
+      <c r="F14" s="50" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G14" s="50" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45308,6 +45464,19 @@
       </c>
       <c r="H14" s="50" t="n"/>
       <c r="I14" s="50" t="n"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="42" t="inlineStr">
@@ -45335,7 +45504,11 @@
           <t>+44-555-111-1111</t>
         </is>
       </c>
-      <c r="F15" s="31" t="n"/>
+      <c r="F15" s="31" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G15" s="31" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45343,6 +45516,19 @@
       </c>
       <c r="H15" s="31" t="n"/>
       <c r="I15" s="31" t="n"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="34" t="inlineStr">
@@ -45397,7 +45583,11 @@
           <t>+1-987-654-3210</t>
         </is>
       </c>
-      <c r="F17" s="31" t="n"/>
+      <c r="F17" s="31" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G17" s="31" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45405,6 +45595,19 @@
       </c>
       <c r="H17" s="31" t="n"/>
       <c r="I17" s="31" t="n"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="34" t="inlineStr">
@@ -45432,7 +45635,11 @@
           <t>+44-123-456-7890</t>
         </is>
       </c>
-      <c r="F18" s="50" t="n"/>
+      <c r="F18" s="50" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G18" s="50" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45440,6 +45647,19 @@
       </c>
       <c r="H18" s="50" t="n"/>
       <c r="I18" s="50" t="n"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="42" t="inlineStr">
@@ -45467,7 +45687,11 @@
           <t>+91-9876543210</t>
         </is>
       </c>
-      <c r="F19" s="31" t="n"/>
+      <c r="F19" s="31" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G19" s="31" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45475,6 +45699,19 @@
       </c>
       <c r="H19" s="31" t="n"/>
       <c r="I19" s="31" t="n"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="34" t="inlineStr">
@@ -45502,7 +45739,11 @@
           <t>+1-555-123-4567</t>
         </is>
       </c>
-      <c r="F20" s="50" t="n"/>
+      <c r="F20" s="50" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G20" s="50" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45510,6 +45751,19 @@
       </c>
       <c r="H20" s="50" t="n"/>
       <c r="I20" s="50" t="n"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="42" t="inlineStr">
@@ -45537,7 +45791,11 @@
           <t>ABC-123-XYZ</t>
         </is>
       </c>
-      <c r="F21" s="31" t="n"/>
+      <c r="F21" s="31" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G21" s="31" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45545,6 +45803,19 @@
       </c>
       <c r="H21" s="31" t="n"/>
       <c r="I21" s="31" t="n"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="34" t="inlineStr">
@@ -45572,7 +45843,11 @@
           <t>+61-123-4567</t>
         </is>
       </c>
-      <c r="F22" s="50" t="n"/>
+      <c r="F22" s="50" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G22" s="50" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45580,6 +45855,19 @@
       </c>
       <c r="H22" s="50" t="n"/>
       <c r="I22" s="50" t="n"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="42" t="inlineStr">
@@ -45607,7 +45895,11 @@
           <t>+1-800-000-0000</t>
         </is>
       </c>
-      <c r="F23" s="31" t="n"/>
+      <c r="F23" s="31" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G23" s="31" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45615,6 +45907,19 @@
       </c>
       <c r="H23" s="31" t="n"/>
       <c r="I23" s="31" t="n"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="34" t="inlineStr">
@@ -45642,7 +45947,11 @@
           <t>+1-800-555-0199</t>
         </is>
       </c>
-      <c r="F24" s="50" t="n"/>
+      <c r="F24" s="50" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G24" s="50" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45650,6 +45959,19 @@
       </c>
       <c r="H24" s="50" t="n"/>
       <c r="I24" s="50" t="n"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="42" t="inlineStr">
@@ -45689,6 +46011,19 @@
       </c>
       <c r="H25" s="31" t="n"/>
       <c r="I25" s="31" t="n"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>State123!</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>POC123!</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="34" t="inlineStr">
@@ -45716,7 +46051,11 @@
           <t>ABC-DEF</t>
         </is>
       </c>
-      <c r="F26" s="50" t="n"/>
+      <c r="F26" s="50" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G26" s="50" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45730,6 +46069,21 @@
       <c r="I26" s="50" t="inlineStr">
         <is>
           <t>ABC</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Ten</t>
         </is>
       </c>
     </row>
@@ -45759,7 +46113,11 @@
           <t>+49-123-456789</t>
         </is>
       </c>
-      <c r="F27" s="31" t="n"/>
+      <c r="F27" s="31" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G27" s="31" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45767,6 +46125,19 @@
       </c>
       <c r="H27" s="31" t="n"/>
       <c r="I27" s="31" t="n"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L27" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="34" t="inlineStr">
@@ -45794,7 +46165,11 @@
           <t>+33-123-456-789</t>
         </is>
       </c>
-      <c r="F28" s="50" t="n"/>
+      <c r="F28" s="50" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G28" s="50" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45802,6 +46177,19 @@
       </c>
       <c r="H28" s="50" t="n"/>
       <c r="I28" s="50" t="n"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L28" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="42" t="inlineStr">
@@ -45829,7 +46217,11 @@
           <t>+34-123-456-789</t>
         </is>
       </c>
-      <c r="F29" s="31" t="n"/>
+      <c r="F29" s="31" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G29" s="31" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45837,6 +46229,19 @@
       </c>
       <c r="H29" s="31" t="n"/>
       <c r="I29" s="31" t="n"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L29" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="34" t="inlineStr">
@@ -45864,7 +46269,11 @@
           <t>+33-123-456-789</t>
         </is>
       </c>
-      <c r="F30" s="50" t="n"/>
+      <c r="F30" s="50" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G30" s="50" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45872,6 +46281,19 @@
       </c>
       <c r="H30" s="50" t="n"/>
       <c r="I30" s="50" t="n"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L30" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="42" t="inlineStr">
@@ -45899,7 +46321,11 @@
           <t>+1-555-222-2222</t>
         </is>
       </c>
-      <c r="F31" s="31" t="n"/>
+      <c r="F31" s="31" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G31" s="31" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45907,6 +46333,19 @@
       </c>
       <c r="H31" s="31" t="n"/>
       <c r="I31" s="31" t="n"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L31" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="34" t="inlineStr">
@@ -45934,7 +46373,11 @@
           <t>+1-555-333-3333</t>
         </is>
       </c>
-      <c r="F32" s="50" t="n"/>
+      <c r="F32" s="50" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G32" s="50" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45944,6 +46387,19 @@
         <v>-5</v>
       </c>
       <c r="I32" s="50" t="n"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L32" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="42" t="inlineStr">
@@ -45971,7 +46427,11 @@
           <t>+1-555-444-4444</t>
         </is>
       </c>
-      <c r="F33" s="31" t="n"/>
+      <c r="F33" s="31" t="inlineStr">
+        <is>
+          <t>123 Tech Park</t>
+        </is>
+      </c>
       <c r="G33" s="31" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45979,6 +46439,19 @@
       </c>
       <c r="H33" s="31" t="n"/>
       <c r="I33" s="31" t="n"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="L33" t="n">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>